<commit_message>
feat(F-NAR-019): polish TREE-DIF-063 xlsx
Alignement xlsx sur merged vocal après re-apply.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-063.xlsx
+++ b/stories/arbres/TREE-DIF-063.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Victorino connaît ce quai, ses bancs, son pigeon. Le fer sent le savon chaud des mains de maman. L'horloge jaune cliquette, sans se presser. Un grain de suie repose sur le ticket rouge. Il est tout petit, papa. Tu le vois, ce grain noir ? Le pigeon penche la tête, près du banc. Le wagon ouvre sa porte, là. Je garde le ticket jusqu'au lac. En ce moment, le sifflet perce le quai. Victorino court trop, le ticket claque. Le grain de suie glisse, presque tombé. Son sourire part, les épaules basses. Tu veux le montrer trop vite ? Papa s'accroupit, à la même hauteur. Merci, tu as ralenti pour le grain.</t>
+          <t>Victorino connaît ce quai, ses bancs, son pigeon. Le fer sent le savon chaud des mains de maman. L'horloge jaune cliquette, sans se presser. Un grain de suie repose sur le ticket rouge. Il est tout petit, papa. Tu le vois, ce grain noir ? Le pigeon penche la tête, près du banc. Le wagon ouvre sa porte, là. Je garde le ticket jusqu'au lac. Le banc du pigeon garde une chaleur ronde. En ce moment, le sifflet perce le quai. Victorino court trop, le ticket claque. Le grain de suie glisse, presque tombé. Son sourire part, les épaules basses. L'envie tape, l'inquiétude aussi, dans la poitrine. Tu veux le montrer trop vite ? Papa s'accroupit, à la même hauteur. Merci, tu as ralenti pour le grain.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino connaît ce quai, ses bancs, son pigeon. Le fer sent le savon chaud des mains de maman. L'horloge jaune cliquette, sans se presser. Un grain de suie repose sur le &lt;emphasis level="moderate"&gt;ticket rouge&lt;/emphasis&gt;. Il est tout petit, papa. Tu le vois, ce grain noir ? Le pigeon penche la tête, près du banc. Le wagon ouvre sa porte, là. Je garde le ticket jusqu'au lac. En ce moment, le sifflet perce le quai. Victorino court trop, le ticket claque. Le grain de suie glisse, presque tombé. Son sourire part, les épaules basses. Tu veux le montrer trop vite ? Papa s'accroupit, à la même hauteur. Merci, tu as ralenti pour le grain.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino connaît ce quai, ses bancs, son pigeon. Le fer sent le savon chaud des mains de maman. L'horloge jaune cliquette, sans se presser. Un grain de suie repose sur le &lt;emphasis level="moderate"&gt;ticket rouge&lt;/emphasis&gt;. Il est tout petit, papa. Tu le vois, ce grain noir ? Le pigeon penche la tête, près du banc. Le wagon ouvre sa porte, là. Je garde le ticket jusqu'au lac. Le banc du pigeon garde une chaleur ronde. En ce moment, le sifflet perce le quai. Victorino court trop, le ticket claque. Le grain de suie glisse, presque tombé. Son sourire part, les épaules basses. L'envie tape, l'inquiétude aussi, dans la poitrine. Tu veux le montrer trop vite ? Papa s'accroupit, à la même hauteur. Merci, tu as ralenti pour le grain.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Victorino connaît ce quai, ses bancs, son pigeon. Le fer sent le savon chaud des mains de maman. L'horloge jaune cliquette, sans se presser. Un grain de suie repose sur le &lt;emphasis&gt;ticket rouge&lt;/emphasis&gt;. Il est tout petit, papa. Tu le vois, ce grain noir ? Le pigeon penche la tête, près du banc. Le wagon ouvre sa porte, là. Je garde le ticket jusqu'au lac. En ce moment, le sifflet perce le quai. Victorino court trop, le ticket claque. Le grain de suie glisse, presque tombé. Son sourire part, les épaules basses. Tu veux le montrer trop vite ? Papa s'accroupit, à la même hauteur. Merci, tu as ralenti pour le grain. [pause]</t>
+          <t>Victorino connaît ce quai, ses bancs, son pigeon. Le fer sent le savon chaud des mains de maman. L'horloge jaune cliquette, sans se presser. Un grain de suie repose sur le &lt;emphasis&gt;ticket rouge&lt;/emphasis&gt;. Il est tout petit, papa. Tu le vois, ce grain noir ? Le pigeon penche la tête, près du banc. Le wagon ouvre sa porte, là. Je garde le ticket jusqu'au lac. Le banc du pigeon garde une chaleur ronde. En ce moment, le sifflet perce le quai. Victorino court trop, le ticket claque. Le grain de suie glisse, presque tombé. Son sourire part, les épaules basses. L'envie tape, l'inquiétude aussi, dans la poitrine. Tu veux le montrer trop vite ? Papa s'accroupit, à la même hauteur. Merci, tu as ralenti pour le grain. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1350,10 +1350,12 @@
 narrateur|Le pigeon penche la tête, près du banc.
 maman|Le wagon ouvre sa porte, là.
 enfant-m|Je garde le ticket jusqu'au lac.
+narrateur|Le banc du pigeon garde une chaleur ronde.
 narrateur|En ce moment, le sifflet perce le quai.
 narrateur|Victorino court trop, le ticket claque.
 narrateur|Le grain de suie glisse, presque tombé.
 narrateur|Son sourire part, les épaules basses.
+narrateur|L'envie tape, l'inquiétude aussi, dans la poitrine.
 papa|Tu veux le montrer trop vite ?
 narrateur|Papa s'accroupit, à la même hauteur.
 papa|Merci, tu as ralenti pour le grain.</t>
@@ -1585,17 +1587,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorino prend le ticket rouge, le grain de suie dessus. Toi, tu vas voir le lac. Il le lève trop haut, trop vite. Le papier claque, le grain penche. Tiens-le bas, près de toi. Victorino baisse le ticket, les joues chaudes. Le sac bleu vient avec nous. Maman glisse la pomme contre sa poche. Les trois, jusqu'au lac. Le grain de suie tient, tout noir. Le ticket est à toi.</t>
+          <t>Victorino prend le ticket rouge, le grain de suie dessus. Toi, tu vas voir le lac. Il le lève trop haut, trop vite. Le papier claque, le grain penche. Tiens-le bas, près de toi. Victorino baisse le ticket, les joues chaudes. Le sac bleu vient avec nous. Maman glisse la pomme contre sa poche. Les trois, jusqu'au lac. Ils marchent vers le wagon du lac. Le grain de suie tient, tout noir. Le ticket est à toi. Le sac et la pomme viennent aussi.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino prend le &lt;emphasis level="moderate"&gt;ticket rouge&lt;/emphasis&gt;, le grain de suie dessus. Toi, tu vas voir le lac. Il le lève trop haut, trop vite. Le papier claque, le grain penche. Tiens-le bas, près de toi. Victorino baisse le ticket, les joues chaudes. Le sac bleu vient avec nous. Maman glisse la pomme contre sa poche. Les trois, jusqu'au lac. Le grain de suie tient, tout noir. Le ticket est à toi.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino prend le &lt;emphasis level="moderate"&gt;ticket rouge&lt;/emphasis&gt;, le grain de suie dessus. Toi, tu vas voir le lac. Il le lève trop haut, trop vite. Le papier claque, le grain penche. Tiens-le bas, près de toi. Victorino baisse le ticket, les joues chaudes. Le sac bleu vient avec nous. Maman glisse la pomme contre sa poche. Les trois, jusqu'au lac. Ils marchent vers le wagon du lac. Le grain de suie tient, tout noir. Le ticket est à toi. Le sac et la pomme viennent aussi.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Victorino prend le &lt;emphasis&gt;ticket rouge&lt;/emphasis&gt;, le grain de suie dessus. Toi, tu vas voir le lac. Il le lève trop haut, trop vite. Le papier claque, le grain penche. Tiens-le bas, près de toi. Victorino baisse le ticket, les joues chaudes. Le sac bleu vient avec nous. Maman glisse la pomme contre sa poche. Les trois, jusqu'au lac. Le grain de suie tient, tout noir. Le ticket est à toi. [pause]</t>
+          <t>Victorino prend le &lt;emphasis&gt;ticket rouge&lt;/emphasis&gt;, le grain de suie dessus. Toi, tu vas voir le lac. Il le lève trop haut, trop vite. Le papier claque, le grain penche. Tiens-le bas, près de toi. Victorino baisse le ticket, les joues chaudes. Le sac bleu vient avec nous. Maman glisse la pomme contre sa poche. Les trois, jusqu'au lac. Ils marchent vers le wagon du lac. Le grain de suie tient, tout noir. Le ticket est à toi. Le sac et la pomme viennent aussi. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1738,8 +1740,10 @@
 papa|Le sac bleu vient avec nous.
 narrateur|Maman glisse la pomme contre sa poche.
 enfant-m|Les trois, jusqu'au lac.
+narrateur|Ils marchent vers le wagon du lac.
 narrateur|Le grain de suie tient, tout noir.
-papa|Le ticket est à toi.</t>
+papa|Le ticket est à toi.
+maman|Le sac et la pomme viennent aussi.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1959,17 +1963,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Dans la main. Oui, tout près. Un sifflet réveille le quai. C'est mon train, pour le lac. Victorino plie un genou, trop vite. Le ticket dessine un pli, le grain penche. On monte ici ? Oui, papa. Le wagon avale leurs pas, un par un.</t>
+          <t>Dans la main. Oui, tout près. Un sifflet réveille le quai. C'est mon train, pour le lac. Victorino plie un genou, trop vite. Le ticket dessine un pli, le grain penche. On monte ici ? Oui, papa. Le wagon avale leurs pas, un par un. Une odeur de fer chaud entre avec eux. On est dedans, Victorino.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans la main. Oui, tout près. Un sifflet réveille le quai. C'est mon train, pour le &lt;emphasis level="moderate"&gt;lac&lt;/emphasis&gt;. Victorino plie un genou, trop vite. Le ticket dessine un pli, le grain penche. On monte ici ? Oui, papa. Le wagon avale leurs pas, un par un.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans la main. Oui, tout près. Un sifflet réveille le quai. C'est mon train, pour le &lt;emphasis level="moderate"&gt;lac&lt;/emphasis&gt;. Victorino plie un genou, trop vite. Le ticket dessine un pli, le grain penche. On monte ici ? Oui, papa. Le wagon avale leurs pas, un par un. Une odeur de fer chaud entre avec eux. On est dedans, Victorino.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Dans la main. Oui, tout près. Un sifflet réveille le quai. C'est mon train, pour le &lt;emphasis&gt;lac&lt;/emphasis&gt;. Victorino plie un genou, trop vite. Le ticket dessine un pli, le grain penche. On monte ici ? Oui, papa. Le wagon avale leurs pas, un par un. [pause]</t>
+          <t>Dans la main. Oui, tout près. Un sifflet réveille le quai. C'est mon train, pour le &lt;emphasis&gt;lac&lt;/emphasis&gt;. Victorino plie un genou, trop vite. Le ticket dessine un pli, le grain penche. On monte ici ? Oui, papa. Le wagon avale leurs pas, un par un. Une odeur de fer chaud entre avec eux. On est dedans, Victorino. [pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2111,7 +2115,9 @@
 narrateur|Le ticket dessine un pli, le grain penche.
 papa|On monte ici ?
 enfant-m|Oui, papa.
-narrateur|Le wagon avale leurs pas, un par un.</t>
+narrateur|Le wagon avale leurs pas, un par un.
+narrateur|Une odeur de fer chaud entre avec eux.
+maman|On est dedans, Victorino.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr">
@@ -2342,17 +2348,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le ticket rouge est tiède. L'allée du wagon file, trop longue. Victorino court vers le fond, pour le lac. Son talon accroche un pli du caoutchouc. Le ticket part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Il regarde le grain de suie, immobile. Tu vois comment, Victorino ?</t>
+          <t>Entre ses doigts, le ticket rouge est tiède. L'allée du wagon file, trop longue. Victorino court vers le fond, pour le lac. Son talon accroche un pli du caoutchouc. Le ticket part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Personne ne donne la réponse. Il écoute les roues, puis le grain. Il regarde le grain de suie, immobile. Tu vois comment, Victorino ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le ticket rouge est tiède. L'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; du wagon file, trop longue. Victorino court vers le fond, pour le lac. Son talon accroche un pli du caoutchouc. Le ticket part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Il regarde le grain de suie, immobile. Tu vois comment, Victorino ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le ticket rouge est tiède. L'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; du wagon file, trop longue. Victorino court vers le fond, pour le lac. Son talon accroche un pli du caoutchouc. Le ticket part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Personne ne donne la réponse. Il écoute les roues, puis le grain. Il regarde le grain de suie, immobile. Tu vois comment, Victorino ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Entre ses doigts, le ticket rouge est tiède. L'&lt;emphasis&gt;allée&lt;/emphasis&gt; du wagon file, trop longue. Victorino court vers le fond, pour le lac. Son talon accroche un pli du caoutchouc. Le ticket part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Il regarde le grain de suie, immobile. Tu vois comment, Victorino ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Entre ses doigts, le ticket rouge est tiède. L'&lt;emphasis&gt;allée&lt;/emphasis&gt; du wagon file, trop longue. Victorino court vers le fond, pour le lac. Son talon accroche un pli du caoutchouc. Le ticket part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Personne ne donne la réponse. Il écoute les roues, puis le grain. Il regarde le grain de suie, immobile. Tu vois comment, Victorino ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -2500,6 +2506,8 @@
 papa|Ici, ce n'est pas le lac.
 narrateur|Papa s'accroupit, à sa hauteur.
 enfant-m|Je ne fonce pas.
+narrateur|Personne ne donne la réponse.
+narrateur|Il écoute les roues, puis le grain.
 narrateur|Il regarde le grain de suie, immobile.
 papa|Tu vois comment, Victorino ?</t>
         </is>
@@ -3840,17 +3848,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Le ticket rouge colle à la vitre froide. Ici, je vois le lac, maman. Dehors, le pré file trop vite. Victorino presse le papier, trop fort. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Le grain de suie reste, seul, sur le rouge.</t>
+          <t>Le ticket rouge colle à la vitre froide. Ici, je vois le lac, maman. Dehors, le pré file trop vite. Victorino presse le papier, trop fort. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Personne ne donne la réponse. Il écoute la vitre, puis le grain. Le grain de suie reste, seul, sur le rouge.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le ticket rouge colle à la &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, maman. Dehors, le pré file trop vite. Victorino presse le papier, trop fort. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Le grain de suie reste, seul, sur le rouge.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le ticket rouge colle à la &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, maman. Dehors, le pré file trop vite. Victorino presse le papier, trop fort. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Personne ne donne la réponse. Il écoute la vitre, puis le grain. Le grain de suie reste, seul, sur le rouge.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le ticket rouge colle à la &lt;emphasis&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, maman. Dehors, le pré file trop vite. Victorino presse le papier, trop fort. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Le grain de suie reste, seul, sur le rouge.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le ticket rouge colle à la &lt;emphasis&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, maman. Dehors, le pré file trop vite. Victorino presse le papier, trop fort. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Personne ne donne la réponse. Il écoute la vitre, puis le grain. Le grain de suie reste, seul, sur le rouge.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -3999,6 +4007,8 @@
 maman|Ce n'est pas le lac, trop tôt.
 narrateur|Maman s'accroupit, à sa hauteur.
 enfant-m|J'attends le grain.
+narrateur|Personne ne donne la réponse.
+narrateur|Il écoute la vitre, puis le grain.
 narrateur|Le grain de suie reste, seul, sur le rouge.</t>
         </is>
       </c>
@@ -5339,17 +5349,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Victorino pose le ticket sur la tablette. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. Le ticket grimpe au bord, trop vite. Il va tomber ! Il veut tout poser d'un coup, pomme et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Il observe le grain de suie, au bord.</t>
+          <t>Victorino pose le ticket sur la tablette. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. Le ticket grimpe au bord, trop vite. Il va tomber ! Il veut tout poser d'un coup, pomme et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Personne ne donne la réponse. Il écoute le bois, puis le grain. Il observe le grain de suie, au bord.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino pose le ticket sur la &lt;emphasis level="moderate"&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. Le ticket grimpe au bord, trop vite. Il va tomber ! Il veut tout poser d'un coup, pomme et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Il observe le grain de suie, au bord.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino pose le ticket sur la &lt;emphasis level="moderate"&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. Le ticket grimpe au bord, trop vite. Il va tomber ! Il veut tout poser d'un coup, pomme et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Personne ne donne la réponse. Il écoute le bois, puis le grain. Il observe le grain de suie, au bord.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Victorino pose le ticket sur la &lt;emphasis&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. Le ticket grimpe au bord, trop vite. Il va tomber ! Il veut tout poser d'un coup, pomme et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Il observe le grain de suie, au bord.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Victorino pose le ticket sur la &lt;emphasis&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. Le ticket grimpe au bord, trop vite. Il va tomber ! Il veut tout poser d'un coup, pomme et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Personne ne donne la réponse. Il écoute le bois, puis le grain. Il observe le grain de suie, au bord.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5498,6 +5508,8 @@
 papa|Trop de choses, trop vite.
 narrateur|Papa s'accroupit, à sa hauteur.
 enfant-m|Je reste.
+narrateur|Personne ne donne la réponse.
+narrateur|Il écoute le bois, puis le grain.
 narrateur|Il observe le grain de suie, au bord.</t>
         </is>
       </c>
@@ -6834,17 +6846,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Victorino passe le sac bleu sous le bras. Tu portes le voyage. Il le lance trop vite, la sangle tourne. Tiens-le contre toi, sans le jeter. La boucle fait un petit clic. Le ticket, ensuite, près de toi. Il glisse la pomme d'une main. Je vais voir le lac. Un genou rebondit, trop pressé. Le ticket reste au bord, le grain visible. Le sac est prêt.</t>
+          <t>Victorino passe le sac bleu sous le bras. Tu portes le voyage. Il le lance trop vite, la sangle tourne. Tiens-le contre toi, sans le jeter. La boucle fait un petit clic. Le ticket, ensuite, près de toi. Il glisse la pomme d'une main. Je vais voir le lac. Un genou rebondit, trop pressé. Ils marchent vers le wagon du lac. Le ticket reste au bord, le grain visible. Le sac est prêt. Le ticket et la pomme viennent aussi.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino passe le &lt;emphasis level="moderate"&gt;sac bleu&lt;/emphasis&gt; sous le bras. Tu portes le voyage. Il le lance trop vite, la sangle tourne. Tiens-le contre toi, sans le jeter. La boucle fait un petit clic. Le ticket, ensuite, près de toi. Il glisse la pomme d'une main. Je vais voir le lac. Un genou rebondit, trop pressé. Le ticket reste au bord, le grain visible. Le sac est prêt.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino passe le &lt;emphasis level="moderate"&gt;sac bleu&lt;/emphasis&gt; sous le bras. Tu portes le voyage. Il le lance trop vite, la sangle tourne. Tiens-le contre toi, sans le jeter. La boucle fait un petit clic. Le ticket, ensuite, près de toi. Il glisse la pomme d'une main. Je vais voir le lac. Un genou rebondit, trop pressé. Ils marchent vers le wagon du lac. Le ticket reste au bord, le grain visible. Le sac est prêt. Le ticket et la pomme viennent aussi.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Victorino passe le &lt;emphasis&gt;sac bleu&lt;/emphasis&gt; sous le bras. Tu portes le voyage. Il le lance trop vite, la sangle tourne. Tiens-le contre toi, sans le jeter. La boucle fait un petit clic. Le ticket, ensuite, près de toi. Il glisse la pomme d'une main. Je vais voir le lac. Un genou rebondit, trop pressé. Le ticket reste au bord, le grain visible. Le sac est prêt. [pause]</t>
+          <t>Victorino passe le &lt;emphasis&gt;sac bleu&lt;/emphasis&gt; sous le bras. Tu portes le voyage. Il le lance trop vite, la sangle tourne. Tiens-le contre toi, sans le jeter. La boucle fait un petit clic. Le ticket, ensuite, près de toi. Il glisse la pomme d'une main. Je vais voir le lac. Un genou rebondit, trop pressé. Ils marchent vers le wagon du lac. Le ticket reste au bord, le grain visible. Le sac est prêt. Le ticket et la pomme viennent aussi. [pause]</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -6987,8 +6999,10 @@
 narrateur|Il glisse la pomme d'une main.
 enfant-m|Je vais voir le lac.
 narrateur|Un genou rebondit, trop pressé.
+narrateur|Ils marchent vers le wagon du lac.
 narrateur|Le ticket reste au bord, le grain visible.
-maman|Le sac est prêt.</t>
+maman|Le sac est prêt.
+papa|Le ticket et la pomme viennent aussi.</t>
         </is>
       </c>
       <c r="AX32" t="inlineStr">
@@ -7204,17 +7218,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Sous le bras. Oui. La boucle du sac chatouille sa manche. C'est mon coin, pour le lac. Victorino secoue le sac, un nuage de laine. Un coin bleu traîne par terre, trop vite. Ça sent le quai tiède. Tes mains, sur le sac ? Oui, papa. Ils montent, le grain de suie contre le bleu.</t>
+          <t>Sous le bras. Oui. La boucle du sac chatouille sa manche. C'est mon coin, pour le lac. Victorino secoue le sac, un nuage de laine. Un coin bleu traîne par terre, trop vite. Ça sent le quai tiède. Tes mains, sur le sac ? Oui, papa. Ils montent, le grain de suie contre le bleu. Une odeur de fer chaud entre avec eux. On est dedans, Victorino.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sous le bras. Oui. La boucle du sac chatouille sa manche. C'est mon coin, pour le &lt;emphasis level="moderate"&gt;lac&lt;/emphasis&gt;. Victorino secoue le sac, un nuage de laine. Un coin bleu traîne par terre, trop vite. Ça sent le quai tiède. Tes mains, sur le sac ? Oui, papa. Ils montent, le grain de suie contre le bleu.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sous le bras. Oui. La boucle du sac chatouille sa manche. C'est mon coin, pour le &lt;emphasis level="moderate"&gt;lac&lt;/emphasis&gt;. Victorino secoue le sac, un nuage de laine. Un coin bleu traîne par terre, trop vite. Ça sent le quai tiède. Tes mains, sur le sac ? Oui, papa. Ils montent, le grain de suie contre le bleu. Une odeur de fer chaud entre avec eux. On est dedans, Victorino.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Sous le bras. Oui. La boucle du sac chatouille sa manche. C'est mon coin, pour le &lt;emphasis&gt;lac&lt;/emphasis&gt;. Victorino secoue le sac, un nuage de laine. Un coin bleu traîne par terre, trop vite. Ça sent le quai tiède. Tes mains, sur le sac ? Oui, papa. Ils montent, le grain de suie contre le bleu. [pause]</t>
+          <t>Sous le bras. Oui. La boucle du sac chatouille sa manche. C'est mon coin, pour le &lt;emphasis&gt;lac&lt;/emphasis&gt;. Victorino secoue le sac, un nuage de laine. Un coin bleu traîne par terre, trop vite. Ça sent le quai tiède. Tes mains, sur le sac ? Oui, papa. Ils montent, le grain de suie contre le bleu. Une odeur de fer chaud entre avec eux. On est dedans, Victorino. [pause]</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7357,7 +7371,9 @@
 maman|Ça sent le quai tiède.
 papa|Tes mains, sur le sac ?
 enfant-m|Oui, papa.
-narrateur|Ils montent, le grain de suie contre le bleu.</t>
+narrateur|Ils montent, le grain de suie contre le bleu.
+narrateur|Une odeur de fer chaud entre avec eux.
+maman|On est dedans, Victorino.</t>
         </is>
       </c>
       <c r="AX34" t="inlineStr">
@@ -7588,17 +7604,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Le sac bleu tape un siège, clic trop fort. L'allée du wagon file, trop étroite. Victorino avance trop vite, le sac en avant. La sangle accroche un dossier, puis lâche. Le sac part trop vite. Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. L'allée n'est pas un chemin de course. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Il cherche le grain de suie, sur le ticket. Le grain est là, contre le bleu.</t>
+          <t>Le sac bleu tape un siège, clic trop fort. L'allée du wagon file, trop étroite. Victorino avance trop vite, le sac en avant. La sangle accroche un dossier, puis lâche. Le sac part trop vite. Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. L'allée n'est pas un chemin de course. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Personne ne donne la réponse. Il écoute les roues, puis le grain. Il cherche le grain de suie, sur le ticket. Le grain est là, contre le bleu.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le sac bleu tape un siège, clic trop fort. L'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; du wagon file, trop étroite. Victorino avance trop vite, le sac en avant. La sangle accroche un dossier, puis lâche. Le sac part trop vite. Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. L'allée n'est pas un chemin de course. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Il cherche le grain de suie, sur le ticket. Le grain est là, contre le bleu.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le sac bleu tape un siège, clic trop fort. L'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; du wagon file, trop étroite. Victorino avance trop vite, le sac en avant. La sangle accroche un dossier, puis lâche. Le sac part trop vite. Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. L'allée n'est pas un chemin de course. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Personne ne donne la réponse. Il écoute les roues, puis le grain. Il cherche le grain de suie, sur le ticket. Le grain est là, contre le bleu.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le sac bleu tape un siège, clic trop fort. L'&lt;emphasis&gt;allée&lt;/emphasis&gt; du wagon file, trop étroite. Victorino avance trop vite, le sac en avant. La sangle accroche un dossier, puis lâche. Le sac part trop vite. Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. L'allée n'est pas un chemin de course. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Il cherche le grain de suie, sur le ticket. Le grain est là, contre le bleu.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le sac bleu tape un siège, clic trop fort. L'&lt;emphasis&gt;allée&lt;/emphasis&gt; du wagon file, trop étroite. Victorino avance trop vite, le sac en avant. La sangle accroche un dossier, puis lâche. Le sac part trop vite. Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. L'allée n'est pas un chemin de course. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Personne ne donne la réponse. Il écoute les roues, puis le grain. Il cherche le grain de suie, sur le ticket. Le grain est là, contre le bleu.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -7746,6 +7762,8 @@
 papa|L'allée n'est pas un chemin de course.
 narrateur|Papa s'accroupit, à sa hauteur.
 enfant-m|Je ne fonce pas.
+narrateur|Personne ne donne la réponse.
+narrateur|Il écoute les roues, puis le grain.
 narrateur|Il cherche le grain de suie, sur le ticket.
 maman|Le grain est là, contre le bleu.</t>
         </is>
@@ -9087,17 +9105,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Victorino pose le sac sous la vitre froide. Ici, je vois le lac, papa. Le sac glisse comme un wagon trop pressé. Une mare passe, trop petite, trop vite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller le sac plus fort, tout de suite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Le grain de suie tient, collé au ticket.</t>
+          <t>Victorino pose le sac sous la vitre froide. Ici, je vois le lac, papa. Le sac glisse comme un wagon trop pressé. Une mare passe, trop petite, trop vite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller le sac plus fort, tout de suite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Personne ne donne la réponse. Il écoute la vitre, puis le grain. Le grain de suie tient, collé au ticket.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino pose le sac sous la &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, papa. Le sac glisse comme un wagon trop pressé. Une mare passe, trop petite, trop vite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller le sac plus fort, tout de suite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Le grain de suie tient, collé au ticket.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino pose le sac sous la &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, papa. Le sac glisse comme un wagon trop pressé. Une mare passe, trop petite, trop vite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller le sac plus fort, tout de suite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Personne ne donne la réponse. Il écoute la vitre, puis le grain. Le grain de suie tient, collé au ticket.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Victorino pose le sac sous la &lt;emphasis&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, papa. Le sac glisse comme un wagon trop pressé. Une mare passe, trop petite, trop vite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller le sac plus fort, tout de suite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Le grain de suie tient, collé au ticket.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Victorino pose le sac sous la &lt;emphasis&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, papa. Le sac glisse comme un wagon trop pressé. Une mare passe, trop petite, trop vite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller le sac plus fort, tout de suite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Personne ne donne la réponse. Il écoute la vitre, puis le grain. Le grain de suie tient, collé au ticket.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -9246,6 +9264,8 @@
 maman|Ce n'est pas le lac, trop tôt.
 narrateur|Maman s'accroupit, à sa hauteur.
 enfant-m|J'attends le grain.
+narrateur|Personne ne donne la réponse.
+narrateur|Il écoute la vitre, puis le grain.
 narrateur|Le grain de suie tient, collé au ticket.</t>
         </is>
       </c>
@@ -10586,17 +10606,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Victorino pousse le sac sur la tablette. Ici, c'est ma table, maman. Le bois plié renvoie chaque secousse. Le sac se faufile sous la tablette, tout seul. Il disparaît ! Il veut tout coincer d'un coup, pomme et ticket. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Il observe le grain de suie, au bord du rouge.</t>
+          <t>Victorino pousse le sac sur la tablette. Ici, c'est ma table, maman. Le bois plié renvoie chaque secousse. Le sac se faufile sous la tablette, tout seul. Il disparaît ! Il veut tout coincer d'un coup, pomme et ticket. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Personne ne donne la réponse. Il écoute le bois, puis le grain. Il observe le grain de suie, au bord du rouge.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino pousse le sac sur la &lt;emphasis level="moderate"&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, maman. Le bois plié renvoie chaque secousse. Le sac se faufile sous la tablette, tout seul. Il disparaît ! Il veut tout coincer d'un coup, pomme et ticket. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Il observe le grain de suie, au bord du rouge.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino pousse le sac sur la &lt;emphasis level="moderate"&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, maman. Le bois plié renvoie chaque secousse. Le sac se faufile sous la tablette, tout seul. Il disparaît ! Il veut tout coincer d'un coup, pomme et ticket. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Personne ne donne la réponse. Il écoute le bois, puis le grain. Il observe le grain de suie, au bord du rouge.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Victorino pousse le sac sur la &lt;emphasis&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, maman. Le bois plié renvoie chaque secousse. Le sac se faufile sous la tablette, tout seul. Il disparaît ! Il veut tout coincer d'un coup, pomme et ticket. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Il observe le grain de suie, au bord du rouge.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Victorino pousse le sac sur la &lt;emphasis&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, maman. Le bois plié renvoie chaque secousse. Le sac se faufile sous la tablette, tout seul. Il disparaît ! Il veut tout coincer d'un coup, pomme et ticket. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Personne ne donne la réponse. Il écoute le bois, puis le grain. Il observe le grain de suie, au bord du rouge.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -10745,6 +10765,8 @@
 papa|Trop de choses, trop vite.
 narrateur|Papa s'accroupit, à sa hauteur.
 enfant-m|Je reste.
+narrateur|Personne ne donne la réponse.
+narrateur|Il écoute le bois, puis le grain.
 narrateur|Il observe le grain de suie, au bord du rouge.</t>
         </is>
       </c>
@@ -12081,17 +12103,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Victorino prend d'abord la pomme. Elle est froide, contre la poche. Garde-la là, près de toi. La peau sent le panier du village. Le ticket et le sac, avec toi. Il les pose près du banc du pigeon. Ma pomme va voyager aussi. Ses talons frappent le quai, trop vite. Le ticket reste visible, le grain de suie dessus. La pomme est prise.</t>
+          <t>Victorino prend d'abord la pomme. Elle est froide, contre la poche. Garde-la là, près de toi. La peau sent le panier du village. Le ticket et le sac, avec toi. Il les pose près du banc du pigeon. Ma pomme va voyager aussi. Ses talons frappent le quai, trop vite. Ils marchent vers le wagon du lac. Le ticket reste visible, le grain de suie dessus. La pomme est prise. Le ticket et le sac viennent aussi.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino prend d'abord la &lt;emphasis level="moderate"&gt;pomme&lt;/emphasis&gt;. Elle est froide, contre la poche. Garde-la là, près de toi. La peau sent le panier du village. Le ticket et le sac, avec toi. Il les pose près du banc du pigeon. Ma pomme va voyager aussi. Ses talons frappent le quai, trop vite. Le ticket reste visible, le grain de suie dessus. La pomme est prise.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino prend d'abord la &lt;emphasis level="moderate"&gt;pomme&lt;/emphasis&gt;. Elle est froide, contre la poche. Garde-la là, près de toi. La peau sent le panier du village. Le ticket et le sac, avec toi. Il les pose près du banc du pigeon. Ma pomme va voyager aussi. Ses talons frappent le quai, trop vite. Ils marchent vers le wagon du lac. Le ticket reste visible, le grain de suie dessus. La pomme est prise. Le ticket et le sac viennent aussi.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Victorino prend d'abord la &lt;emphasis&gt;pomme&lt;/emphasis&gt;. Elle est froide, contre la poche. Garde-la là, près de toi. La peau sent le panier du village. Le ticket et le sac, avec toi. Il les pose près du banc du pigeon. Ma pomme va voyager aussi. Ses talons frappent le quai, trop vite. Le ticket reste visible, le grain de suie dessus. La pomme est prise. [pause]</t>
+          <t>Victorino prend d'abord la &lt;emphasis&gt;pomme&lt;/emphasis&gt;. Elle est froide, contre la poche. Garde-la là, près de toi. La peau sent le panier du village. Le ticket et le sac, avec toi. Il les pose près du banc du pigeon. Ma pomme va voyager aussi. Ses talons frappent le quai, trop vite. Ils marchent vers le wagon du lac. Le ticket reste visible, le grain de suie dessus. La pomme est prise. Le ticket et le sac viennent aussi. [pause]</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -12233,8 +12255,10 @@
 narrateur|Il les pose près du banc du pigeon.
 enfant-m|Ma pomme va voyager aussi.
 narrateur|Ses talons frappent le quai, trop vite.
+narrateur|Ils marchent vers le wagon du lac.
 narrateur|Le ticket reste visible, le grain de suie dessus.
-papa|La pomme est prise.</t>
+papa|La pomme est prise.
+maman|Le ticket et le sac viennent aussi.</t>
         </is>
       </c>
       <c r="AX60" t="inlineStr">
@@ -12450,17 +12474,17 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Dans la poche. Oui. La pomme roule un peu, puis s'arrête. Elle voyage contre moi. Victorino la serre, la lâche, la reprend. Un reflet rouge frotte sa poche. Le wagon est prêt, devant. On y va, tous les trois ? Oui. Ils montent, la pomme froide, le grain noir.</t>
+          <t>Dans la poche. Oui. La pomme roule un peu, puis s'arrête. Elle voyage contre moi. Victorino la serre, la lâche, la reprend. Un reflet rouge frotte sa poche. Le wagon est prêt, devant. On y va, tous les trois ? Oui. Ils montent, la pomme froide, le grain noir. Une odeur de fer chaud entre avec eux. On est dedans, Victorino.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans la poche. Oui. La pomme roule un peu, puis s'arrête. Elle voyage contre moi. Victorino la serre, la lâche, la reprend. Un reflet rouge frotte sa poche. Le wagon est prêt, devant. On y va, tous les trois ? Oui. Ils montent, la pomme froide, le grain noir.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans la poche. Oui. La pomme roule un peu, puis s'arrête. Elle voyage contre moi. Victorino la serre, la lâche, la reprend. Un reflet rouge frotte sa poche. Le wagon est prêt, devant. On y va, tous les trois ? Oui. Ils montent, la pomme froide, le grain noir. Une odeur de fer chaud entre avec eux. On est dedans, Victorino.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Dans la poche. Oui. La pomme roule un peu, puis s'arrête. Elle voyage contre moi. Victorino la serre, la lâche, la reprend. Un reflet rouge frotte sa poche. Le wagon est prêt, devant. On y va, tous les trois ? Oui. Ils montent, la pomme froide, le grain noir. [pause]</t>
+          <t>Dans la poche. Oui. La pomme roule un peu, puis s'arrête. Elle voyage contre moi. Victorino la serre, la lâche, la reprend. Un reflet rouge frotte sa poche. Le wagon est prêt, devant. On y va, tous les trois ? Oui. Ils montent, la pomme froide, le grain noir. Une odeur de fer chaud entre avec eux. On est dedans, Victorino. [pause]</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -12603,7 +12627,9 @@
 maman|Le wagon est prêt, devant.
 papa|On y va, tous les trois ?
 enfant-m|Oui.
-narrateur|Ils montent, la pomme froide, le grain noir.</t>
+narrateur|Ils montent, la pomme froide, le grain noir.
+narrateur|Une odeur de fer chaud entre avec eux.
+maman|On est dedans, Victorino.</t>
         </is>
       </c>
       <c r="AX62" t="inlineStr">
@@ -12834,17 +12860,17 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>La pomme tape sa poche, trop haut. L'allée du wagon file, trop longue. Victorino court vers le fond, la pomme qui rebondit. Son talon accroche un pli du caoutchouc. Ma pomme part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Il regarde le grain de suie, sur le ticket. Le grain reste, lui.</t>
+          <t>La pomme tape sa poche, trop haut. L'allée du wagon file, trop longue. Victorino court vers le fond, la pomme qui rebondit. Son talon accroche un pli du caoutchouc. Ma pomme part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Personne ne donne la réponse. Il écoute les roues, puis le grain. Il regarde le grain de suie, sur le ticket. Le grain reste, lui.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La pomme tape sa poche, trop haut. L'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; du wagon file, trop longue. Victorino court vers le fond, la pomme qui rebondit. Son talon accroche un pli du caoutchouc. Ma pomme part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Il regarde le grain de suie, sur le ticket. Le grain reste, lui.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La pomme tape sa poche, trop haut. L'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; du wagon file, trop longue. Victorino court vers le fond, la pomme qui rebondit. Son talon accroche un pli du caoutchouc. Ma pomme part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Personne ne donne la réponse. Il écoute les roues, puis le grain. Il regarde le grain de suie, sur le ticket. Le grain reste, lui.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;La pomme tape sa poche, trop haut. L'&lt;emphasis&gt;allée&lt;/emphasis&gt; du wagon file, trop longue. Victorino court vers le fond, la pomme qui rebondit. Son talon accroche un pli du caoutchouc. Ma pomme part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Il regarde le grain de suie, sur le ticket. Le grain reste, lui.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;La pomme tape sa poche, trop haut. L'&lt;emphasis&gt;allée&lt;/emphasis&gt; du wagon file, trop longue. Victorino court vers le fond, la pomme qui rebondit. Son talon accroche un pli du caoutchouc. Ma pomme part ! Les roues changent de rythme, plus dures. Son sourire part, la poitrine serrée. Ici, ce n'est pas le lac. Papa s'accroupit, à sa hauteur. Je ne fonce pas. Personne ne donne la réponse. Il écoute les roues, puis le grain. Il regarde le grain de suie, sur le ticket. Le grain reste, lui.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -12992,6 +13018,8 @@
 papa|Ici, ce n'est pas le lac.
 narrateur|Papa s'accroupit, à sa hauteur.
 enfant-m|Je ne fonce pas.
+narrateur|Personne ne donne la réponse.
+narrateur|Il écoute les roues, puis le grain.
 narrateur|Il regarde le grain de suie, sur le ticket.
 maman|Le grain reste, lui.</t>
         </is>
@@ -14333,17 +14361,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Victorino pose la pomme contre la vitre froide. Ici, je vois le lac, maman. La pomme file, une bosse après l'autre. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller la pomme plus fort, trop vite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Le grain de suie reste, seul, sur le rouge.</t>
+          <t>Victorino pose la pomme contre la vitre froide. Ici, je vois le lac, maman. La pomme file, une bosse après l'autre. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller la pomme plus fort, trop vite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Personne ne donne la réponse. Il écoute la vitre, puis le grain. Le grain de suie reste, seul, sur le rouge.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino pose la pomme contre la &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, maman. La pomme file, une bosse après l'autre. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller la pomme plus fort, trop vite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Le grain de suie reste, seul, sur le rouge.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino pose la pomme contre la &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, maman. La pomme file, une bosse après l'autre. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller la pomme plus fort, trop vite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Personne ne donne la réponse. Il écoute la vitre, puis le grain. Le grain de suie reste, seul, sur le rouge.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Victorino pose la pomme contre la &lt;emphasis&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, maman. La pomme file, une bosse après l'autre. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller la pomme plus fort, trop vite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Le grain de suie reste, seul, sur le rouge.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Victorino pose la pomme contre la &lt;emphasis&gt;vitre&lt;/emphasis&gt; froide. Ici, je vois le lac, maman. La pomme file, une bosse après l'autre. Une mare passe, trop petite. L'eau, je l'ai vue ! Un éclair plus large frappe le verre. Il veut coller la pomme plus fort, trop vite. Son sourire part, la poitrine serrée. Ce n'est pas le lac, trop tôt. Maman s'accroupit, à sa hauteur. J'attends le grain. Personne ne donne la réponse. Il écoute la vitre, puis le grain. Le grain de suie reste, seul, sur le rouge.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -14492,6 +14520,8 @@
 maman|Ce n'est pas le lac, trop tôt.
 narrateur|Maman s'accroupit, à sa hauteur.
 enfant-m|J'attends le grain.
+narrateur|Personne ne donne la réponse.
+narrateur|Il écoute la vitre, puis le grain.
 narrateur|Le grain de suie reste, seul, sur le rouge.</t>
         </is>
       </c>
@@ -15832,17 +15862,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Victorino pose la pomme sur la tablette. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. La pomme disparaît vers le bord, trop loin. Elle va tomber ! Il veut tout poser d'un coup, ticket et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Il observe le grain de suie, au bord du ticket.</t>
+          <t>Victorino pose la pomme sur la tablette. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. La pomme disparaît vers le bord, trop loin. Elle va tomber ! Il veut tout poser d'un coup, ticket et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Personne ne donne la réponse. Il écoute le bois, puis le grain. Il observe le grain de suie, au bord du ticket.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino pose la pomme sur la &lt;emphasis level="moderate"&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. La pomme disparaît vers le bord, trop loin. Elle va tomber ! Il veut tout poser d'un coup, ticket et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Il observe le grain de suie, au bord du ticket.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino pose la pomme sur la &lt;emphasis level="moderate"&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. La pomme disparaît vers le bord, trop loin. Elle va tomber ! Il veut tout poser d'un coup, ticket et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Personne ne donne la réponse. Il écoute le bois, puis le grain. Il observe le grain de suie, au bord du ticket.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Victorino pose la pomme sur la &lt;emphasis&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. La pomme disparaît vers le bord, trop loin. Elle va tomber ! Il veut tout poser d'un coup, ticket et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Il observe le grain de suie, au bord du ticket.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Victorino pose la pomme sur la &lt;emphasis&gt;tablette&lt;/emphasis&gt;. Ici, c'est ma table, papa. Le bois plié renvoie chaque secousse. La pomme disparaît vers le bord, trop loin. Elle va tomber ! Il veut tout poser d'un coup, ticket et sac. La tablette saute plus fort, trop chargée. Son sourire part, la poitrine serrée. Trop de choses, trop vite. Papa s'accroupit, à sa hauteur. Je reste. Personne ne donne la réponse. Il écoute le bois, puis le grain. Il observe le grain de suie, au bord du ticket.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -15991,6 +16021,8 @@
 papa|Trop de choses, trop vite.
 narrateur|Papa s'accroupit, à sa hauteur.
 enfant-m|Je reste.
+narrateur|Personne ne donne la réponse.
+narrateur|Il écoute le bois, puis le grain.
 narrateur|Il observe le grain de suie, au bord du ticket.</t>
         </is>
       </c>
@@ -17321,7 +17353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17378,6 +17410,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>